<commit_message>
docs: refresh public README and strategy evidence
</commit_message>
<xml_diff>
--- a/reports/forward_test_report.xlsx
+++ b/reports/forward_test_report.xlsx
@@ -11,13 +11,17 @@
     <sheet name="Standard Limit Real Tick" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Forward Trades" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Forward Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Telegram Delivery" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Forward Exit Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Strategy Policy" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Telegram Delivery" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Standard Limit Real Tick'!$A$1:$Z$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Forward Trades'!$A$1:$S$315</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Forward Summary'!$A$1:$H$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Telegram Delivery'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Forward Summary'!$A$1:$N$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Forward Exit Summary'!$A$1:$F$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Strategy Policy'!$A$1:$P$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Telegram Delivery'!$A$1:$D$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -459,7 +463,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-16 12:25:41 WIB</t>
+          <t>2026-07-16 13:26:44 WIB</t>
         </is>
       </c>
     </row>
@@ -490,22 +494,46 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Telegram evidence</t>
+          <t>Strategy policy</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Delivery journal is populated only after TELEGRAM_EVENT_LOG_ENABLED is enabled locally.</t>
+          <t>Deployment status is based on the published forward evidence and configured entry-path policy.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Exit evidence</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Soft TP, server TP, SL, and unmatched exit comments are summarized separately for payoff review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Telegram evidence</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Delivery journal is populated only after TELEGRAM_EVENT_LOG_ENABLED is enabled locally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Warning</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Results are historical evidence, not a profit guarantee or trading recommendation.</t>
         </is>
@@ -29406,7 +29434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -29416,7 +29444,13 @@
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -29457,7 +29491,37 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
+          <t>gross_profit_usd</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>gross_loss_usd</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>avg_win_usd</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>avg_loss_usd</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
           <t>net_profit_usd</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>profit_factor</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>payoff_ratio</t>
         </is>
       </c>
     </row>
@@ -29490,7 +29554,25 @@
         <v>66.67</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2899999999999991</v>
+        <v>30.3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>30.01</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="K2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="3">
@@ -29522,7 +29604,25 @@
         <v>40</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1899999999999995</v>
+        <v>28.49</v>
+      </c>
+      <c r="I3" t="n">
+        <v>28.68</v>
+      </c>
+      <c r="J3" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="K3" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1.49</v>
       </c>
     </row>
     <row r="4">
@@ -29556,6 +29656,24 @@
       <c r="H4" t="n">
         <v>13.64</v>
       </c>
+      <c r="I4" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="K4" t="n">
+        <v/>
+      </c>
+      <c r="L4" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="M4" t="n">
+        <v/>
+      </c>
+      <c r="N4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -29588,6 +29706,24 @@
       <c r="H5" t="n">
         <v>14.29</v>
       </c>
+      <c r="I5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="K5" t="n">
+        <v/>
+      </c>
+      <c r="L5" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="M5" t="n">
+        <v/>
+      </c>
+      <c r="N5" t="n">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -29618,7 +29754,25 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>35.17</v>
+      </c>
+      <c r="J6" t="n">
+        <v/>
+      </c>
+      <c r="K6" t="n">
+        <v>17.58</v>
+      </c>
+      <c r="L6" t="n">
         <v>-35.17</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -29650,7 +29804,25 @@
         <v>60</v>
       </c>
       <c r="H7" t="n">
+        <v>64.48</v>
+      </c>
+      <c r="I7" t="n">
+        <v>46.71</v>
+      </c>
+      <c r="J7" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="K7" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="L7" t="n">
         <v>17.77</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.92</v>
       </c>
     </row>
     <row r="8">
@@ -29682,7 +29854,25 @@
         <v>40</v>
       </c>
       <c r="H8" t="n">
+        <v>45.69</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="J8" t="n">
+        <v>22.85</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L8" t="n">
         <v>39.98</v>
+      </c>
+      <c r="M8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N8" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -29714,7 +29904,25 @@
         <v>75</v>
       </c>
       <c r="H9" t="n">
+        <v>61.46</v>
+      </c>
+      <c r="I9" t="n">
+        <v>27.61</v>
+      </c>
+      <c r="J9" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="K9" t="n">
+        <v>27.61</v>
+      </c>
+      <c r="L9" t="n">
         <v>33.85</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.74</v>
       </c>
     </row>
     <row r="10">
@@ -29746,7 +29954,25 @@
         <v>39.44</v>
       </c>
       <c r="H10" t="n">
-        <v>-17.23999999999999</v>
+        <v>271.41</v>
+      </c>
+      <c r="I10" t="n">
+        <v>288.65</v>
+      </c>
+      <c r="J10" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="K10" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-17.24</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1.44</v>
       </c>
     </row>
     <row r="11">
@@ -29778,7 +30004,25 @@
         <v>38.46</v>
       </c>
       <c r="H11" t="n">
-        <v>-98.39999999999999</v>
+        <v>94.93000000000001</v>
+      </c>
+      <c r="I11" t="n">
+        <v>193.33</v>
+      </c>
+      <c r="J11" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="K11" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-98.40000000000001</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.79</v>
       </c>
     </row>
     <row r="12">
@@ -29810,7 +30054,25 @@
         <v>68.97</v>
       </c>
       <c r="H12" t="n">
-        <v>-63.98999999999999</v>
+        <v>93.13</v>
+      </c>
+      <c r="I12" t="n">
+        <v>157.12</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="K12" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-63.99</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.27</v>
       </c>
     </row>
     <row r="13">
@@ -29842,7 +30104,25 @@
         <v>68.75</v>
       </c>
       <c r="H13" t="n">
+        <v>142.01</v>
+      </c>
+      <c r="I13" t="n">
+        <v>63.14</v>
+      </c>
+      <c r="J13" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="K13" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="L13" t="n">
         <v>78.87</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1.02</v>
       </c>
     </row>
     <row r="14">
@@ -29874,7 +30154,25 @@
         <v>75</v>
       </c>
       <c r="H14" t="n">
+        <v>58.84</v>
+      </c>
+      <c r="I14" t="n">
+        <v>47.97</v>
+      </c>
+      <c r="J14" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="K14" t="n">
+        <v>23.98</v>
+      </c>
+      <c r="L14" t="n">
         <v>10.87</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.41</v>
       </c>
     </row>
     <row r="15">
@@ -29906,7 +30204,25 @@
         <v>50</v>
       </c>
       <c r="H15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="L15" t="n">
         <v>0.74</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1.42</v>
       </c>
     </row>
     <row r="16">
@@ -29938,7 +30254,25 @@
         <v>33.33</v>
       </c>
       <c r="H16" t="n">
+        <v>15.77</v>
+      </c>
+      <c r="I16" t="n">
+        <v>35.89</v>
+      </c>
+      <c r="J16" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="K16" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="L16" t="n">
         <v>-20.12</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.88</v>
       </c>
     </row>
     <row r="17">
@@ -29972,6 +30306,24 @@
       <c r="H17" t="n">
         <v>15.4</v>
       </c>
+      <c r="I17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="K17" t="n">
+        <v/>
+      </c>
+      <c r="L17" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="M17" t="n">
+        <v/>
+      </c>
+      <c r="N17" t="n">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -30002,7 +30354,25 @@
         <v>61.54</v>
       </c>
       <c r="H18" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="I18" t="n">
+        <v>72.72</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="K18" t="n">
+        <v>14.54</v>
+      </c>
+      <c r="L18" t="n">
         <v>-32.44</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="19">
@@ -30036,6 +30406,24 @@
       <c r="H19" t="n">
         <v>9.640000000000001</v>
       </c>
+      <c r="I19" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="K19" t="n">
+        <v/>
+      </c>
+      <c r="L19" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="M19" t="n">
+        <v/>
+      </c>
+      <c r="N19" t="n">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -30066,7 +30454,25 @@
         <v>53.57</v>
       </c>
       <c r="H20" t="n">
+        <v>209.79</v>
+      </c>
+      <c r="I20" t="n">
+        <v>377.04</v>
+      </c>
+      <c r="J20" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="K20" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="L20" t="n">
         <v>-167.25</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="21">
@@ -30098,7 +30504,25 @@
         <v>71.43000000000001</v>
       </c>
       <c r="H21" t="n">
+        <v>41.22</v>
+      </c>
+      <c r="I21" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="L21" t="n">
         <v>17.72</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="22">
@@ -30130,11 +30554,29 @@
         <v>86.67</v>
       </c>
       <c r="H22" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I22" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="J22" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="K22" t="n">
+        <v>19.19</v>
+      </c>
+      <c r="L22" t="n">
         <v>113.03</v>
       </c>
+      <c r="M22" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.61</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H22"/>
+  <autoFilter ref="A1:N22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -30145,18 +30587,2848 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>entry_type</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>timeframe</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>exit_type</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>trades</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>net_profit_usd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.81</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-19.76</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15.24</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>28.29</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-28.48</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>13.64</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>14.29</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-35.17</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>48.15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-41.71</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11.33</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-1.92</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-3.79</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>45.69</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>43.61</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-27.61</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>17.85</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>70</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-32.06999999999999</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>14.83</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>30</v>
+      </c>
+      <c r="F21" t="n">
+        <v>31.11</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-129.51</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>22</v>
+      </c>
+      <c r="F23" t="n">
+        <v>57.14</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-145.79</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" t="n">
+        <v>24.66</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>44.35</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-43.94</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>78.46000000000001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>OTHER_OR_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-47.97</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>45.34</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OTHER_OR_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-29.32</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-2.52</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-3.28</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SND</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>SND</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>OTHER_OR_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-26.31</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-7.390000000000001</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>6</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-13.74</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BPR</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>9.640000000000001</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>31</v>
+      </c>
+      <c r="F44" t="n">
+        <v>-5.429999999999998</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>12</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-293.68</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>13</v>
+      </c>
+      <c r="F46" t="n">
+        <v>131.86</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>11</v>
+      </c>
+      <c r="F47" t="n">
+        <v>3.43</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>10</v>
+      </c>
+      <c r="F48" t="n">
+        <v>14.29</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SOFT_TP</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>5</v>
+      </c>
+      <c r="F49" t="n">
+        <v>16.51</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>4</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-32.72</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TAKE_PROFIT</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>6</v>
+      </c>
+      <c r="F51" t="n">
+        <v>129.24</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F51"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>entry_type</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>timeframe</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>trades</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>wins</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>losses</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>winrate_pct</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>gross_profit_usd</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>gross_loss_usd</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>avg_win_usd</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>avg_loss_usd</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>net_profit_usd</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>profit_factor</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>payoff_ratio</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>policy_reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="H2" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>30.01</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="K2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>No automatic promotion; keep evaluating forward profit factor and payoff ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H3" t="n">
+        <v>28.49</v>
+      </c>
+      <c r="I3" t="n">
+        <v>28.68</v>
+      </c>
+      <c r="J3" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="K3" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>No automatic promotion; keep evaluating forward profit factor and payoff ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="K4" t="n">
+        <v/>
+      </c>
+      <c r="L4" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="M4" t="n">
+        <v/>
+      </c>
+      <c r="N4" t="n">
+        <v/>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>No automatic promotion; keep evaluating forward profit factor and payoff ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="K5" t="n">
+        <v/>
+      </c>
+      <c r="L5" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="M5" t="n">
+        <v/>
+      </c>
+      <c r="N5" t="n">
+        <v/>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>No automatic promotion; keep evaluating forward profit factor and payoff ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>35.17</v>
+      </c>
+      <c r="J6" t="n">
+        <v/>
+      </c>
+      <c r="K6" t="n">
+        <v>17.58</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-35.17</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v/>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Forward sample is small and currently negative; replay is required before reconsideration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>60</v>
+      </c>
+      <c r="H7" t="n">
+        <v>64.48</v>
+      </c>
+      <c r="I7" t="n">
+        <v>46.71</v>
+      </c>
+      <c r="J7" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="K7" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="L7" t="n">
+        <v>17.77</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>No automatic promotion; keep evaluating forward profit factor and payoff ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>40</v>
+      </c>
+      <c r="H8" t="n">
+        <v>45.69</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="J8" t="n">
+        <v>22.85</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L8" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="M8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N8" t="n">
+        <v>12</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>No automatic promotion; keep evaluating forward profit factor and payoff ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Standard Limit</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>75</v>
+      </c>
+      <c r="H9" t="n">
+        <v>61.46</v>
+      </c>
+      <c r="I9" t="n">
+        <v>27.61</v>
+      </c>
+      <c r="J9" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="K9" t="n">
+        <v>27.61</v>
+      </c>
+      <c r="L9" t="n">
+        <v>33.85</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>No automatic promotion; keep evaluating forward profit factor and payoff ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>71</v>
+      </c>
+      <c r="E10" t="n">
+        <v>28</v>
+      </c>
+      <c r="F10" t="n">
+        <v>43</v>
+      </c>
+      <c r="G10" t="n">
+        <v>39.44</v>
+      </c>
+      <c r="H10" t="n">
+        <v>271.41</v>
+      </c>
+      <c r="I10" t="n">
+        <v>288.65</v>
+      </c>
+      <c r="J10" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="K10" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-17.24</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>39</v>
+      </c>
+      <c r="E11" t="n">
+        <v>15</v>
+      </c>
+      <c r="F11" t="n">
+        <v>24</v>
+      </c>
+      <c r="G11" t="n">
+        <v>38.46</v>
+      </c>
+      <c r="H11" t="n">
+        <v>94.93000000000001</v>
+      </c>
+      <c r="I11" t="n">
+        <v>193.33</v>
+      </c>
+      <c r="J11" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="K11" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-98.40000000000001</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>29</v>
+      </c>
+      <c r="E12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" t="n">
+        <v>68.97</v>
+      </c>
+      <c r="H12" t="n">
+        <v>93.13</v>
+      </c>
+      <c r="I12" t="n">
+        <v>157.12</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="K12" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-63.99</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>68.75</v>
+      </c>
+      <c r="H13" t="n">
+        <v>142.01</v>
+      </c>
+      <c r="I13" t="n">
+        <v>63.14</v>
+      </c>
+      <c r="J13" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="K13" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="L13" t="n">
+        <v>78.87</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Restricted candidate needs at least 30 resolved forward trades before promotion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H14" t="n">
+        <v>58.84</v>
+      </c>
+      <c r="I14" t="n">
+        <v>47.97</v>
+      </c>
+      <c r="J14" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="K14" t="n">
+        <v>23.98</v>
+      </c>
+      <c r="L14" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>50</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="H16" t="n">
+        <v>15.77</v>
+      </c>
+      <c r="I16" t="n">
+        <v>35.89</v>
+      </c>
+      <c r="J16" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="K16" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-20.12</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SND</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
+      </c>
+      <c r="H17" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="K17" t="n">
+        <v/>
+      </c>
+      <c r="L17" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="M17" t="n">
+        <v/>
+      </c>
+      <c r="N17" t="n">
+        <v/>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>13</v>
+      </c>
+      <c r="E18" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>61.54</v>
+      </c>
+      <c r="H18" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="I18" t="n">
+        <v>72.72</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="K18" t="n">
+        <v>14.54</v>
+      </c>
+      <c r="L18" t="n">
+        <v>-32.44</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BPR</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>100</v>
+      </c>
+      <c r="H19" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="K19" t="n">
+        <v/>
+      </c>
+      <c r="L19" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="M19" t="n">
+        <v/>
+      </c>
+      <c r="N19" t="n">
+        <v/>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FVG</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>56</v>
+      </c>
+      <c r="E20" t="n">
+        <v>30</v>
+      </c>
+      <c r="F20" t="n">
+        <v>26</v>
+      </c>
+      <c r="G20" t="n">
+        <v>53.57</v>
+      </c>
+      <c r="H20" t="n">
+        <v>209.79</v>
+      </c>
+      <c r="I20" t="n">
+        <v>377.04</v>
+      </c>
+      <c r="J20" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="K20" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="L20" t="n">
+        <v>-167.25</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>21</v>
+      </c>
+      <c r="E21" t="n">
+        <v>15</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="H21" t="n">
+        <v>41.22</v>
+      </c>
+      <c r="I21" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="L21" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Instant WatchZone is limited to the forward-positive OB M30/H1 candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>WatchZone</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>M30</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>15</v>
+      </c>
+      <c r="E22" t="n">
+        <v>13</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="n">
+        <v>86.67</v>
+      </c>
+      <c r="H22" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I22" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="J22" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="K22" t="n">
+        <v>19.19</v>
+      </c>
+      <c r="L22" t="n">
+        <v>113.03</v>
+      </c>
+      <c r="M22" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Restricted candidate needs at least 30 resolved forward trades before promotion.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
           <t>sent_at_wib</t>
         </is>
       </c>
@@ -30176,8 +33448,29 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-16T13:25:59+07:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>🧹 &lt;b&gt;[Risk Management] Cleaned up 1 zombie pending orders:&lt;/b&gt;
+• Order #66666 (SL violated)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:D2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>